<commit_message>
Updated country service dataset, fixed UI picker layout, and added issue tracking Excel log to docs
</commit_message>
<xml_diff>
--- a/CountryExplorer/docs/CountryExplorer_API_Status_Codes.xlsx
+++ b/CountryExplorer/docs/CountryExplorer_API_Status_Codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\CountryExplorer\CountryExplorer\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3F0C9B-72C3-4E65-AB63-3B61A254553E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2135E1FF-A28D-4898-8C11-3A354E1EFE04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8148" yWindow="144" windowWidth="14892" windowHeight="11592" xr2:uid="{76559FE1-15A7-40B4-B041-3321AEE415FF}"/>
   </bookViews>
@@ -115,7 +115,7 @@
     </font>
     <font>
       <sz val="16"/>
-      <color theme="0"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -130,7 +130,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="-0.249977111117893"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -152,10 +152,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -535,12 +535,12 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="7" spans="2:5" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">

</xml_diff>